<commit_message>
Update expense tracker - 6/4/2026, 11:51:54 pm
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -872,7 +872,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="2" t="str">
-        <v>2026-03-01</v>
+        <v>2026-02-28</v>
       </c>
       <c r="C5" s="2" t="str">
         <v>Bought Email Domain from Godaddy</v>
@@ -952,34 +952,34 @@
         <v>120</v>
       </c>
       <c r="H6" s="2" t="str">
-        <v>INR</v>
+        <v>USD</v>
       </c>
       <c r="I6" s="2">
+        <v>10080</v>
+      </c>
+      <c r="J6" s="2">
         <v>120</v>
-      </c>
-      <c r="J6" s="2">
-        <v>1.4285714285714286</v>
       </c>
       <c r="K6" s="2">
         <v>120</v>
       </c>
       <c r="L6" s="2" t="str">
-        <v>INR</v>
+        <v>USD</v>
       </c>
       <c r="M6" s="2">
+        <v>10080</v>
+      </c>
+      <c r="N6" s="2">
         <v>120</v>
-      </c>
-      <c r="N6" s="2">
-        <v>1.4285714285714286</v>
       </c>
       <c r="O6" s="2">
         <v>50</v>
       </c>
       <c r="P6" s="2">
-        <v>60</v>
+        <v>5040</v>
       </c>
       <c r="Q6" s="2">
-        <v>60</v>
+        <v>5040</v>
       </c>
       <c r="R6" s="2">
         <v>0</v>

</xml_diff>

<commit_message>
Update expense tracker - 6/4/2026, 11:53:07 pm
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -798,7 +798,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:T6"/>
+  <dimension ref="A2:T7"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -991,9 +991,71 @@
         <v>84</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>2026-02-20</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Bought Web domain from goDaddy</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>Software / Tools</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>Piyal</v>
+      </c>
+      <c r="G7" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="H7" s="2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I7" s="2">
+        <v>1906.8</v>
+      </c>
+      <c r="J7" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="K7" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="L7" s="2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="M7" s="2">
+        <v>1906.8</v>
+      </c>
+      <c r="N7" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="O7" s="2">
+        <v>50</v>
+      </c>
+      <c r="P7" s="2">
+        <v>953.4</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>953.4</v>
+      </c>
+      <c r="R7" s="2">
+        <v>0</v>
+      </c>
+      <c r="S7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T7" s="2">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:T6"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:T7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update expense tracker - 7/4/2026, 12:06:54 am
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -410,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:E42"/>
+  <dimension ref="A2:E43"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -514,7 +514,7 @@
         <v/>
       </c>
       <c r="C15" s="2" t="str">
-        <v>Software / Tools</v>
+        <v>Legal / Admin</v>
       </c>
     </row>
     <row r="16">
@@ -525,7 +525,7 @@
         <v/>
       </c>
       <c r="C16" s="2" t="str">
-        <v>Marketing</v>
+        <v>Travel &amp; Refreshments</v>
       </c>
     </row>
     <row r="17">
@@ -536,7 +536,7 @@
         <v/>
       </c>
       <c r="C17" s="2" t="str">
-        <v>Legal / Admin</v>
+        <v>Miscellaneous</v>
       </c>
     </row>
     <row r="18">
@@ -547,7 +547,7 @@
         <v/>
       </c>
       <c r="C18" s="2" t="str">
-        <v>Travel &amp; Refreshments</v>
+        <v>Budgeted</v>
       </c>
     </row>
     <row r="19">
@@ -558,7 +558,7 @@
         <v/>
       </c>
       <c r="C19" s="2" t="str">
-        <v>Miscellaneous</v>
+        <v>Invoiced</v>
       </c>
     </row>
     <row r="20">
@@ -569,7 +569,7 @@
         <v/>
       </c>
       <c r="C20" s="2" t="str">
-        <v>Budgeted</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="21">
@@ -580,7 +580,7 @@
         <v/>
       </c>
       <c r="C21" s="2" t="str">
-        <v>Invoiced</v>
+        <v>Cancelled</v>
       </c>
     </row>
     <row r="22">
@@ -591,7 +591,7 @@
         <v/>
       </c>
       <c r="C22" s="2" t="str">
-        <v>Paid</v>
+        <v>Budgeted</v>
       </c>
     </row>
     <row r="23">
@@ -602,7 +602,7 @@
         <v/>
       </c>
       <c r="C23" s="2" t="str">
-        <v>Cancelled</v>
+        <v>Invoiced</v>
       </c>
     </row>
     <row r="24">
@@ -613,7 +613,7 @@
         <v/>
       </c>
       <c r="C24" s="2" t="str">
-        <v>Budgeted</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="25">
@@ -624,7 +624,7 @@
         <v/>
       </c>
       <c r="C25" s="2" t="str">
-        <v>Invoiced</v>
+        <v>Cancelled</v>
       </c>
     </row>
     <row r="26">
@@ -635,7 +635,7 @@
         <v/>
       </c>
       <c r="C26" s="2" t="str">
-        <v>Paid</v>
+        <v>Cancelled</v>
       </c>
     </row>
     <row r="27">
@@ -646,7 +646,7 @@
         <v/>
       </c>
       <c r="C27" s="2" t="str">
-        <v>Cancelled</v>
+        <v>Budgeted</v>
       </c>
     </row>
     <row r="28">
@@ -657,7 +657,7 @@
         <v/>
       </c>
       <c r="C28" s="2" t="str">
-        <v>Cancelled</v>
+        <v>Invoiced</v>
       </c>
     </row>
     <row r="29">
@@ -668,7 +668,7 @@
         <v/>
       </c>
       <c r="C29" s="2" t="str">
-        <v>Budgeted</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="30">
@@ -679,7 +679,7 @@
         <v/>
       </c>
       <c r="C30" s="2" t="str">
-        <v>Invoiced</v>
+        <v>Cancelled</v>
       </c>
     </row>
     <row r="31">
@@ -690,7 +690,7 @@
         <v/>
       </c>
       <c r="C31" s="2" t="str">
-        <v>Paid</v>
+        <v>Cancelled</v>
       </c>
     </row>
     <row r="32">
@@ -701,7 +701,7 @@
         <v/>
       </c>
       <c r="C32" s="2" t="str">
-        <v>Cancelled</v>
+        <v>Budgeted</v>
       </c>
     </row>
     <row r="35">
@@ -720,7 +720,7 @@
         <v/>
       </c>
       <c r="C36" s="2" t="str">
-        <v>Cancelled</v>
+        <v>Invoiced</v>
       </c>
     </row>
     <row r="37">
@@ -731,7 +731,7 @@
         <v/>
       </c>
       <c r="C37" s="2" t="str">
-        <v>Budgeted</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="38">
@@ -742,7 +742,7 @@
         <v/>
       </c>
       <c r="C38" s="2" t="str">
-        <v>Invoiced</v>
+        <v>Cancelled</v>
       </c>
     </row>
     <row r="39">
@@ -753,7 +753,7 @@
         <v/>
       </c>
       <c r="C39" s="2" t="str">
-        <v>Paid</v>
+        <v>Cancelled</v>
       </c>
     </row>
     <row r="40">
@@ -764,7 +764,7 @@
         <v/>
       </c>
       <c r="C40" s="2" t="str">
-        <v>Cancelled</v>
+        <v>Budgeted</v>
       </c>
     </row>
     <row r="41">
@@ -775,7 +775,7 @@
         <v/>
       </c>
       <c r="C41" s="2" t="str">
-        <v>Cancelled</v>
+        <v>Invoiced</v>
       </c>
     </row>
     <row r="42">
@@ -786,19 +786,30 @@
         <v/>
       </c>
       <c r="C42" s="2" t="str">
-        <v>Budgeted</v>
+        <v>Paid</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B43" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C43" s="2" t="str">
+        <v>Cancelled</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:E42"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:E43"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:T7"/>
+  <dimension ref="A2:T4"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -867,195 +878,9 @@
         <v>Rate Used</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>1</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>2026-02-28</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <v>Bought Email Domain from Godaddy</v>
-      </c>
-      <c r="D5" s="2" t="str">
-        <v>Software / Tools</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <v>Paid</v>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v>Piyal</v>
-      </c>
-      <c r="G5" s="2">
-        <v>1656</v>
-      </c>
-      <c r="H5" s="2" t="str">
-        <v>INR</v>
-      </c>
-      <c r="I5" s="2">
-        <v>1656</v>
-      </c>
-      <c r="J5" s="2">
-        <v>19.714285714285715</v>
-      </c>
-      <c r="K5" s="2">
-        <v>1656</v>
-      </c>
-      <c r="L5" s="2" t="str">
-        <v>INR</v>
-      </c>
-      <c r="M5" s="2">
-        <v>1656</v>
-      </c>
-      <c r="N5" s="2">
-        <v>19.714285714285715</v>
-      </c>
-      <c r="O5" s="2">
-        <v>50</v>
-      </c>
-      <c r="P5" s="2">
-        <v>828</v>
-      </c>
-      <c r="Q5" s="2">
-        <v>828</v>
-      </c>
-      <c r="R5" s="2">
-        <v>0</v>
-      </c>
-      <c r="S5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T5" s="2">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>2</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>2026-02-19</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>Legal Fees for Company Formation</v>
-      </c>
-      <c r="D6" s="2" t="str">
-        <v>Software / Tools</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>Paid</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>Gautham</v>
-      </c>
-      <c r="G6" s="2">
-        <v>120</v>
-      </c>
-      <c r="H6" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="I6" s="2">
-        <v>10080</v>
-      </c>
-      <c r="J6" s="2">
-        <v>120</v>
-      </c>
-      <c r="K6" s="2">
-        <v>120</v>
-      </c>
-      <c r="L6" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="M6" s="2">
-        <v>10080</v>
-      </c>
-      <c r="N6" s="2">
-        <v>120</v>
-      </c>
-      <c r="O6" s="2">
-        <v>50</v>
-      </c>
-      <c r="P6" s="2">
-        <v>5040</v>
-      </c>
-      <c r="Q6" s="2">
-        <v>5040</v>
-      </c>
-      <c r="R6" s="2">
-        <v>0</v>
-      </c>
-      <c r="S6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T6" s="2">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>3</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>2026-02-20</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>Bought Web domain from goDaddy</v>
-      </c>
-      <c r="D7" s="2" t="str">
-        <v>Software / Tools</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>Paid</v>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v>Piyal</v>
-      </c>
-      <c r="G7" s="2">
-        <v>22.7</v>
-      </c>
-      <c r="H7" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="I7" s="2">
-        <v>1906.8</v>
-      </c>
-      <c r="J7" s="2">
-        <v>22.7</v>
-      </c>
-      <c r="K7" s="2">
-        <v>22.7</v>
-      </c>
-      <c r="L7" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="M7" s="2">
-        <v>1906.8</v>
-      </c>
-      <c r="N7" s="2">
-        <v>22.7</v>
-      </c>
-      <c r="O7" s="2">
-        <v>50</v>
-      </c>
-      <c r="P7" s="2">
-        <v>953.4</v>
-      </c>
-      <c r="Q7" s="2">
-        <v>953.4</v>
-      </c>
-      <c r="R7" s="2">
-        <v>0</v>
-      </c>
-      <c r="S7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T7" s="2">
-        <v>84</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:T7"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:T4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update expense tracker - 7/4/2026, 12:42:46 am
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -410,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:E43"/>
+  <dimension ref="A2:E17"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -436,7 +436,7 @@
         <v>USD→INR</v>
       </c>
       <c r="C5" s="2">
-        <v>84</v>
+        <v>93.13</v>
       </c>
     </row>
     <row r="8">
@@ -506,310 +506,24 @@
         <v>🏷️ Categories</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C15" s="2" t="str">
-        <v>Legal / Admin</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C16" s="2" t="str">
-        <v>Travel &amp; Refreshments</v>
-      </c>
-    </row>
     <row r="17">
       <c r="A17" s="2" t="str">
         <v/>
       </c>
       <c r="B17" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C17" s="2" t="str">
-        <v>Miscellaneous</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C18" s="2" t="str">
-        <v>Budgeted</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C19" s="2" t="str">
-        <v>Invoiced</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B20" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C20" s="2" t="str">
-        <v>Paid</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B21" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C21" s="2" t="str">
-        <v>Cancelled</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B22" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C22" s="2" t="str">
-        <v>Budgeted</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B23" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C23" s="2" t="str">
-        <v>Invoiced</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B24" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C24" s="2" t="str">
-        <v>Paid</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B25" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C25" s="2" t="str">
-        <v>Cancelled</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B26" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C26" s="2" t="str">
-        <v>Cancelled</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B27" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C27" s="2" t="str">
-        <v>Budgeted</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B28" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C28" s="2" t="str">
-        <v>Invoiced</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B29" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C29" s="2" t="str">
-        <v>Paid</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B30" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C30" s="2" t="str">
-        <v>Cancelled</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B31" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C31" s="2" t="str">
-        <v>Cancelled</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B32" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C32" s="2" t="str">
-        <v>Budgeted</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B35" s="2" t="str">
         <v>🔄 Stages</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B36" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C36" s="2" t="str">
-        <v>Invoiced</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B37" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C37" s="2" t="str">
-        <v>Paid</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B38" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C38" s="2" t="str">
-        <v>Cancelled</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B39" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C39" s="2" t="str">
-        <v>Cancelled</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B40" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C40" s="2" t="str">
-        <v>Budgeted</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B41" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C41" s="2" t="str">
-        <v>Invoiced</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B42" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C42" s="2" t="str">
-        <v>Paid</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B43" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C43" s="2" t="str">
-        <v>Cancelled</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:E43"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:E17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:T4"/>
+  <dimension ref="A2:U4"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -877,10 +591,13 @@
       <c r="T4" s="2" t="str">
         <v>Rate Used</v>
       </c>
+      <c r="U4" s="2" t="str">
+        <v>Expense ID</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:T4"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:U4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update expense tracker - 7/4/2026, 12:51:52 am
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -410,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:E17"/>
+  <dimension ref="A2:E26"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -506,24 +506,123 @@
         <v>🏷️ Categories</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B15" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C15" s="2" t="str">
+        <v>Software / Tools</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B16" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C16" s="2" t="str">
+        <v>Marketing</v>
+      </c>
+    </row>
     <row r="17">
       <c r="A17" s="2" t="str">
         <v/>
       </c>
       <c r="B17" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C17" s="2" t="str">
+        <v>Legal / Admin</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B18" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C18" s="2" t="str">
+        <v>Travel &amp; Refreshments</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B19" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C19" s="2" t="str">
+        <v>Miscellaneous</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B22" s="2" t="str">
         <v>🔄 Stages</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B23" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C23" s="2" t="str">
+        <v>Budgeted</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B24" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C24" s="2" t="str">
+        <v>Invoiced</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B25" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C25" s="2" t="str">
+        <v>Paid</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B26" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C26" s="2" t="str">
+        <v>Cancelled</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:E17"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:E26"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:U4"/>
+  <dimension ref="A2:U5"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -595,9 +694,74 @@
         <v>Expense ID</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>2026-02-19</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>Company formation fees with CT Gov</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v>Software / Tools</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>Piyal</v>
+      </c>
+      <c r="G5" s="2">
+        <v>120</v>
+      </c>
+      <c r="H5" s="2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I5" s="2">
+        <v>11175.599999999999</v>
+      </c>
+      <c r="J5" s="2">
+        <v>119.99999999999999</v>
+      </c>
+      <c r="K5" s="2">
+        <v>120</v>
+      </c>
+      <c r="L5" s="2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="M5" s="2">
+        <v>11175.599999999999</v>
+      </c>
+      <c r="N5" s="2">
+        <v>119.99999999999999</v>
+      </c>
+      <c r="O5" s="2">
+        <v>50</v>
+      </c>
+      <c r="P5" s="2">
+        <v>5587.799999999999</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>5587.799999999999</v>
+      </c>
+      <c r="R5" s="2">
+        <v>0</v>
+      </c>
+      <c r="S5" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T5" s="2">
+        <v>93.13</v>
+      </c>
+      <c r="U5" s="2">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:U4"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:U5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update expense tracker - 7/4/2026, 12:53:20 am
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -622,7 +622,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:U5"/>
+  <dimension ref="A2:U6"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -705,7 +705,7 @@
         <v>Company formation fees with CT Gov</v>
       </c>
       <c r="D5" s="2" t="str">
-        <v>Software / Tools</v>
+        <v>Legal / Admin</v>
       </c>
       <c r="E5" s="2" t="str">
         <v>Paid</v>
@@ -759,9 +759,74 @@
         <v>1</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>2</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>2026-04-06</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>Web Domain Bought from GoDaddy</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v>Software / Tools</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>Piyal</v>
+      </c>
+      <c r="G6" s="2">
+        <v>25</v>
+      </c>
+      <c r="H6" s="2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I6" s="2">
+        <v>2328.25</v>
+      </c>
+      <c r="J6" s="2">
+        <v>25</v>
+      </c>
+      <c r="K6" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="L6" s="2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="M6" s="2">
+        <v>2114.051</v>
+      </c>
+      <c r="N6" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="O6" s="2">
+        <v>50</v>
+      </c>
+      <c r="P6" s="2">
+        <v>1057.0255</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>1057.0255</v>
+      </c>
+      <c r="R6" s="2">
+        <v>-214.19900000000007</v>
+      </c>
+      <c r="S6" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T6" s="2">
+        <v>93.13</v>
+      </c>
+      <c r="U6" s="2">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:U5"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:U6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update expense tracker - 7/4/2026, 12:54:36 am
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -622,7 +622,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:U6"/>
+  <dimension ref="A2:U7"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -824,9 +824,74 @@
         <v>2</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Email Domain Bought from GoDaddy</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>Software / Tools</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>Piyal</v>
+      </c>
+      <c r="G7" s="2">
+        <v>20</v>
+      </c>
+      <c r="H7" s="2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I7" s="2">
+        <v>1862.6</v>
+      </c>
+      <c r="J7" s="2">
+        <v>20</v>
+      </c>
+      <c r="K7" s="2">
+        <v>19.71</v>
+      </c>
+      <c r="L7" s="2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="M7" s="2">
+        <v>1835.5923</v>
+      </c>
+      <c r="N7" s="2">
+        <v>19.71</v>
+      </c>
+      <c r="O7" s="2">
+        <v>50</v>
+      </c>
+      <c r="P7" s="2">
+        <v>917.79615</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>917.79615</v>
+      </c>
+      <c r="R7" s="2">
+        <v>-27.007699999999886</v>
+      </c>
+      <c r="S7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T7" s="2">
+        <v>93.13</v>
+      </c>
+      <c r="U7" s="2">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:U6"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:U7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update expense tracker - 7/4/2026, 12:56:36 am
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -514,7 +514,7 @@
         <v/>
       </c>
       <c r="C15" s="2" t="str">
-        <v>Software / Tools</v>
+        <v>Legal / Admin</v>
       </c>
     </row>
     <row r="16">
@@ -525,7 +525,7 @@
         <v/>
       </c>
       <c r="C16" s="2" t="str">
-        <v>Marketing</v>
+        <v>Travel &amp; Refreshments</v>
       </c>
     </row>
     <row r="17">
@@ -536,7 +536,7 @@
         <v/>
       </c>
       <c r="C17" s="2" t="str">
-        <v>Legal / Admin</v>
+        <v>Miscellaneous</v>
       </c>
     </row>
     <row r="18">
@@ -547,7 +547,7 @@
         <v/>
       </c>
       <c r="C18" s="2" t="str">
-        <v>Travel &amp; Refreshments</v>
+        <v>Budgeted</v>
       </c>
     </row>
     <row r="19">
@@ -558,26 +558,29 @@
         <v/>
       </c>
       <c r="C19" s="2" t="str">
-        <v>Miscellaneous</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B22" s="2" t="str">
-        <v>🔄 Stages</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B23" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C23" s="2" t="str">
-        <v>Budgeted</v>
+        <v>Invoiced</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B20" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C20" s="2" t="str">
+        <v>Paid</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C21" s="2" t="str">
+        <v>Cancelled</v>
       </c>
     </row>
     <row r="24">
@@ -585,10 +588,7 @@
         <v/>
       </c>
       <c r="B24" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C24" s="2" t="str">
-        <v>Invoiced</v>
+        <v>🔄 Stages</v>
       </c>
     </row>
     <row r="25">
@@ -622,7 +622,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:U7"/>
+  <dimension ref="A2:U4"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -694,204 +694,9 @@
         <v>Expense ID</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>1</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>2026-02-19</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <v>Company formation fees with CT Gov</v>
-      </c>
-      <c r="D5" s="2" t="str">
-        <v>Legal / Admin</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <v>Paid</v>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v>Piyal</v>
-      </c>
-      <c r="G5" s="2">
-        <v>120</v>
-      </c>
-      <c r="H5" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="I5" s="2">
-        <v>11175.599999999999</v>
-      </c>
-      <c r="J5" s="2">
-        <v>119.99999999999999</v>
-      </c>
-      <c r="K5" s="2">
-        <v>120</v>
-      </c>
-      <c r="L5" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="M5" s="2">
-        <v>11175.599999999999</v>
-      </c>
-      <c r="N5" s="2">
-        <v>119.99999999999999</v>
-      </c>
-      <c r="O5" s="2">
-        <v>50</v>
-      </c>
-      <c r="P5" s="2">
-        <v>5587.799999999999</v>
-      </c>
-      <c r="Q5" s="2">
-        <v>5587.799999999999</v>
-      </c>
-      <c r="R5" s="2">
-        <v>0</v>
-      </c>
-      <c r="S5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T5" s="2">
-        <v>93.13</v>
-      </c>
-      <c r="U5" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>2</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>2026-04-06</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>Web Domain Bought from GoDaddy</v>
-      </c>
-      <c r="D6" s="2" t="str">
-        <v>Software / Tools</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>Paid</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>Piyal</v>
-      </c>
-      <c r="G6" s="2">
-        <v>25</v>
-      </c>
-      <c r="H6" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="I6" s="2">
-        <v>2328.25</v>
-      </c>
-      <c r="J6" s="2">
-        <v>25</v>
-      </c>
-      <c r="K6" s="2">
-        <v>22.7</v>
-      </c>
-      <c r="L6" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="M6" s="2">
-        <v>2114.051</v>
-      </c>
-      <c r="N6" s="2">
-        <v>22.7</v>
-      </c>
-      <c r="O6" s="2">
-        <v>50</v>
-      </c>
-      <c r="P6" s="2">
-        <v>1057.0255</v>
-      </c>
-      <c r="Q6" s="2">
-        <v>1057.0255</v>
-      </c>
-      <c r="R6" s="2">
-        <v>-214.19900000000007</v>
-      </c>
-      <c r="S6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T6" s="2">
-        <v>93.13</v>
-      </c>
-      <c r="U6" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>3</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>2026-03-01</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>Email Domain Bought from GoDaddy</v>
-      </c>
-      <c r="D7" s="2" t="str">
-        <v>Software / Tools</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>Paid</v>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v>Piyal</v>
-      </c>
-      <c r="G7" s="2">
-        <v>20</v>
-      </c>
-      <c r="H7" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="I7" s="2">
-        <v>1862.6</v>
-      </c>
-      <c r="J7" s="2">
-        <v>20</v>
-      </c>
-      <c r="K7" s="2">
-        <v>19.71</v>
-      </c>
-      <c r="L7" s="2" t="str">
-        <v>USD</v>
-      </c>
-      <c r="M7" s="2">
-        <v>1835.5923</v>
-      </c>
-      <c r="N7" s="2">
-        <v>19.71</v>
-      </c>
-      <c r="O7" s="2">
-        <v>50</v>
-      </c>
-      <c r="P7" s="2">
-        <v>917.79615</v>
-      </c>
-      <c r="Q7" s="2">
-        <v>917.79615</v>
-      </c>
-      <c r="R7" s="2">
-        <v>-27.007699999999886</v>
-      </c>
-      <c r="S7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T7" s="2">
-        <v>93.13</v>
-      </c>
-      <c r="U7" s="2">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:U7"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:U4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update expense tracker - 7/4/2026, 1:15:59 am
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -410,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:E26"/>
+  <dimension ref="A2:E17"/>
   <sheetData>
     <row r="2">
       <c r="A2" s="2" t="str">
@@ -506,116 +506,17 @@
         <v>🏷️ Categories</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C15" s="2" t="str">
-        <v>Legal / Admin</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C16" s="2" t="str">
-        <v>Travel &amp; Refreshments</v>
-      </c>
-    </row>
     <row r="17">
       <c r="A17" s="2" t="str">
         <v/>
       </c>
       <c r="B17" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C17" s="2" t="str">
-        <v>Miscellaneous</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C18" s="2" t="str">
-        <v>Budgeted</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C19" s="2" t="str">
-        <v>Invoiced</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B20" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C20" s="2" t="str">
-        <v>Paid</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B21" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C21" s="2" t="str">
-        <v>Cancelled</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B24" s="2" t="str">
         <v>🔄 Stages</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B25" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C25" s="2" t="str">
-        <v>Paid</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B26" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C26" s="2" t="str">
-        <v>Cancelled</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:E26"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:E17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update expense tracker - 7/4/2026, 1:20:37 am
</commit_message>
<xml_diff>
--- a/expense.xlsx
+++ b/expense.xlsx
@@ -410,8 +410,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:E17"/>
+  <dimension ref="A1:F40"/>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E1" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F1" s="2" t="str">
+        <v/>
+      </c>
+    </row>
     <row r="2">
       <c r="A2" s="2" t="str">
         <v/>
@@ -419,6 +439,38 @@
       <c r="B2" s="2" t="str">
         <v>⚙️ Kneuralabs Settings</v>
       </c>
+      <c r="C2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="str">
@@ -427,6 +479,18 @@
       <c r="B4" s="2" t="str">
         <v>💱 Exchange Rate</v>
       </c>
+      <c r="C4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="str">
@@ -435,8 +499,57 @@
       <c r="B5" s="2" t="str">
         <v>USD→INR</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C6" s="2">
         <v>93.13</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -444,7 +557,19 @@
         <v/>
       </c>
       <c r="B8" s="2" t="str">
-        <v>👥 Partners</v>
+        <v/>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -452,16 +577,19 @@
         <v/>
       </c>
       <c r="B9" s="2" t="str">
-        <v>ID</v>
+        <v>👥 Partners</v>
       </c>
       <c r="C9" s="2" t="str">
-        <v>Name</v>
+        <v/>
       </c>
       <c r="D9" s="2" t="str">
-        <v>Currency</v>
+        <v/>
       </c>
       <c r="E9" s="2" t="str">
-        <v>Split %</v>
+        <v/>
+      </c>
+      <c r="F9" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -469,16 +597,19 @@
         <v/>
       </c>
       <c r="B10" s="2" t="str">
-        <v>P1</v>
+        <v>ID</v>
       </c>
       <c r="C10" s="2" t="str">
-        <v>Piyal</v>
+        <v>Name</v>
       </c>
       <c r="D10" s="2" t="str">
-        <v>INR</v>
-      </c>
-      <c r="E10" s="2">
-        <v>50</v>
+        <v>Currency</v>
+      </c>
+      <c r="E10" s="2" t="str">
+        <v>Split %</v>
+      </c>
+      <c r="F10" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -486,24 +617,119 @@
         <v/>
       </c>
       <c r="B11" s="2" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="C11" s="2" t="str">
-        <v>Gautham</v>
+        <v>Piyal</v>
       </c>
       <c r="D11" s="2" t="str">
-        <v>USD</v>
+        <v>INR</v>
       </c>
       <c r="E11" s="2">
         <v>50</v>
       </c>
+      <c r="F11" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B12" s="2" t="str">
+        <v>P2</v>
+      </c>
+      <c r="C12" s="2" t="str">
+        <v>Gautham</v>
+      </c>
+      <c r="D12" s="2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="E12" s="2">
+        <v>50</v>
+      </c>
+      <c r="F12" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B13" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C13" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D13" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E13" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F13" s="2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="str">
         <v/>
       </c>
       <c r="B14" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C14" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D14" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E14" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F14" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B15" s="2" t="str">
         <v>🏷️ Categories</v>
+      </c>
+      <c r="C15" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D15" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E15" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F15" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B16" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C16" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D16" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E16" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F16" s="2" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -511,12 +737,484 @@
         <v/>
       </c>
       <c r="B17" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C17" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D17" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E17" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F17" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B18" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C18" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D18" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E18" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F18" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B19" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C19" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D19" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E19" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F19" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B20" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C20" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D20" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E20" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F20" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C21" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D21" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E21" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F21" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B22" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C22" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D22" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E22" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F22" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B23" s="2" t="str">
         <v>🔄 Stages</v>
+      </c>
+      <c r="C23" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D23" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E23" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F23" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B24" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C24" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D24" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E24" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F24" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B25" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C25" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D25" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E25" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F25" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B26" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C26" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D26" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E26" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F26" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B27" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C27" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D27" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E27" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F27" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B28" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C28" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D28" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E28" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F28" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B29" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C29" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D29" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E29" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F29" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B30" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C30" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D30" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E30" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F30" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B31" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C31" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D31" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E31" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F31" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F32" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F33" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B34" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C34" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D34" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E34" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F34" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B35" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C35" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D35" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E35" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F35" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B36" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C36" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D36" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E36" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F36" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B37" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C37" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D37" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E37" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F37" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B38" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C38" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D38" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E38" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F38" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B39" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C39" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D39" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E39" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F39" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B40" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C40" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D40" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E40" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F40" s="2" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A2:E17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F40"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>